<commit_message>
feat(import): style excel upload template headers
</commit_message>
<xml_diff>
--- a/frontend/werkzeuge-import-muster.xlsx
+++ b/frontend/werkzeuge-import-muster.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K2"/>
   <cols>
     <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="40.83203125" customWidth="1"/>
@@ -412,7 +412,7 @@
     <col min="11" max="11" width="34.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" t="str">
         <v>Werkzeug</v>
       </c>
@@ -445,11 +445,46 @@
       </c>
       <c r="K1" t="str">
         <v>Wartungsnotiz</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>